<commit_message>
se arreglaron datos de biomasa, hay que volver a correr notebooks creados antes de preparing_data
</commit_message>
<xml_diff>
--- a/fermentation_model/data/Laboratorio 2026/Vendimia_2026/mosto_natural_xthiol.xlsx
+++ b/fermentation_model/data/Laboratorio 2026/Vendimia_2026/mosto_natural_xthiol.xlsx
@@ -19858,7 +19858,7 @@
         <v>1050.7</v>
       </c>
       <c r="F5" s="5">
-        <v>17.899999999999999</v>
+        <v>34.8</v>
       </c>
       <c r="G5" s="5"/>
       <c r="H5" s="5">
@@ -20943,9 +20943,7 @@
       <c r="E11" s="5">
         <v>998.8</v>
       </c>
-      <c r="F11" s="5">
-        <v>28.96</v>
-      </c>
+      <c r="F11" s="5"/>
       <c r="G11" s="5"/>
       <c r="H11" s="5">
         <v>0.46</v>
@@ -21013,12 +21011,8 @@
       </c>
       <c r="AL11" s="3"/>
       <c r="AM11" s="3"/>
-      <c r="AN11" s="3">
-        <v>31.26</v>
-      </c>
-      <c r="AO11" s="3">
-        <v>5.65</v>
-      </c>
+      <c r="AN11" s="3"/>
+      <c r="AO11" s="3"/>
       <c r="AP11" s="3">
         <v>6.65</v>
       </c>
@@ -22221,7 +22215,7 @@
         <v>1050.3</v>
       </c>
       <c r="F18" s="5">
-        <v>31.72</v>
+        <v>51.92</v>
       </c>
       <c r="G18" s="5"/>
       <c r="H18" s="5">
@@ -23306,9 +23300,7 @@
       <c r="E24" s="5">
         <v>999.5</v>
       </c>
-      <c r="F24" s="5">
-        <v>35.33</v>
-      </c>
+      <c r="F24" s="5"/>
       <c r="G24" s="5"/>
       <c r="H24" s="5">
         <v>0.67</v>
@@ -23376,12 +23368,8 @@
       </c>
       <c r="AL24" s="3"/>
       <c r="AM24" s="3"/>
-      <c r="AN24" s="3">
-        <v>36.409999999999997</v>
-      </c>
-      <c r="AO24" s="3">
-        <v>8.23</v>
-      </c>
+      <c r="AN24" s="3"/>
+      <c r="AO24" s="3"/>
       <c r="AP24" s="3">
         <v>8.1999999999999993</v>
       </c>
@@ -24584,7 +24572,7 @@
         <v>1058.3</v>
       </c>
       <c r="F31" s="5">
-        <v>14.9</v>
+        <v>30.65</v>
       </c>
       <c r="G31" s="5"/>
       <c r="H31" s="5">
@@ -24654,10 +24642,10 @@
       <c r="AL31" s="3"/>
       <c r="AM31" s="3"/>
       <c r="AN31" s="3">
-        <v>32.869999999999997</v>
+        <v>36.56</v>
       </c>
       <c r="AO31" s="3">
-        <v>22.66</v>
+        <v>23.53</v>
       </c>
       <c r="AP31" s="3">
         <v>129.96</v>
@@ -25472,9 +25460,7 @@
       <c r="E36" s="5">
         <v>1016.1</v>
       </c>
-      <c r="F36" s="5">
-        <v>41.09</v>
-      </c>
+      <c r="F36" s="5"/>
       <c r="G36" s="5">
         <v>8.8000000000000078E-2</v>
       </c>
@@ -25544,12 +25530,8 @@
       </c>
       <c r="AL36" s="3"/>
       <c r="AM36" s="3"/>
-      <c r="AN36" s="3">
-        <v>43.01</v>
-      </c>
-      <c r="AO36" s="3">
-        <v>10</v>
-      </c>
+      <c r="AN36" s="3"/>
+      <c r="AO36" s="3"/>
       <c r="AP36" s="3">
         <v>43.21</v>
       </c>
@@ -28575,9 +28557,7 @@
       <c r="E55" s="5">
         <v>995.6</v>
       </c>
-      <c r="F55" s="5">
-        <v>29.88</v>
-      </c>
+      <c r="F55" s="5"/>
       <c r="G55" s="5">
         <v>9.220000000000006E-2</v>
       </c>
@@ -28651,12 +28631,8 @@
       <c r="AM55" s="3">
         <v>1.31</v>
       </c>
-      <c r="AN55" s="3">
-        <v>41.32</v>
-      </c>
-      <c r="AO55" s="3">
-        <v>5.39</v>
-      </c>
+      <c r="AN55" s="3"/>
+      <c r="AO55" s="3"/>
       <c r="AP55" s="3">
         <v>0.01</v>
       </c>
@@ -30578,9 +30554,7 @@
       <c r="E68" s="5">
         <v>994.5</v>
       </c>
-      <c r="F68" s="5">
-        <v>20.43</v>
-      </c>
+      <c r="F68" s="5"/>
       <c r="G68" s="5">
         <v>0.10299999999999976</v>
       </c>
@@ -30654,12 +30628,8 @@
       <c r="AM68" s="3">
         <v>1.71</v>
       </c>
-      <c r="AN68" s="3">
-        <v>31.26</v>
-      </c>
-      <c r="AO68" s="3">
-        <v>6.14</v>
-      </c>
+      <c r="AN68" s="3"/>
+      <c r="AO68" s="3"/>
       <c r="AP68" s="3">
         <v>0</v>
       </c>
@@ -32436,9 +32406,7 @@
       <c r="E80" s="5">
         <v>995.8</v>
       </c>
-      <c r="F80" s="5">
-        <v>4.6100000000000003</v>
-      </c>
+      <c r="F80" s="5"/>
       <c r="G80" s="5">
         <v>0.10789999999999988</v>
       </c>
@@ -32512,12 +32480,8 @@
       <c r="AM80" s="3">
         <v>1.83</v>
       </c>
-      <c r="AN80" s="3">
-        <v>6.76</v>
-      </c>
-      <c r="AO80" s="3">
-        <v>0</v>
-      </c>
+      <c r="AN80" s="3"/>
+      <c r="AO80" s="3"/>
       <c r="AP80" s="3">
         <v>0.02</v>
       </c>
@@ -37223,7 +37187,7 @@
         <v>35.71</v>
       </c>
       <c r="H5" s="3">
-        <v>17.899999999999999</v>
+        <v>34.8</v>
       </c>
       <c r="I5" s="3">
         <v>17.2</v>
@@ -37631,15 +37595,9 @@
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
-      <c r="G11" s="3">
-        <v>31.26</v>
-      </c>
-      <c r="H11" s="3">
-        <v>28.96</v>
-      </c>
-      <c r="I11" s="3">
-        <v>5.65</v>
-      </c>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
       <c r="J11" s="3">
         <v>6.65</v>
       </c>
@@ -38111,7 +38069,7 @@
         <v>52.69</v>
       </c>
       <c r="H18" s="3">
-        <v>31.72</v>
+        <v>51.92</v>
       </c>
       <c r="I18" s="3">
         <v>19.100000000000001</v>
@@ -38519,15 +38477,9 @@
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
-      <c r="G24" s="3">
-        <v>36.409999999999997</v>
-      </c>
-      <c r="H24" s="3">
-        <v>35.33</v>
-      </c>
-      <c r="I24" s="3">
-        <v>8.23</v>
-      </c>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
       <c r="J24" s="3">
         <v>8.1999999999999993</v>
       </c>
@@ -38996,13 +38948,13 @@
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
       <c r="G31" s="3">
-        <v>32.869999999999997</v>
+        <v>36.56</v>
       </c>
       <c r="H31" s="3">
-        <v>14.9</v>
+        <v>30.65</v>
       </c>
       <c r="I31" s="3">
-        <v>22.66</v>
+        <v>23.53</v>
       </c>
       <c r="J31" s="3">
         <v>129.96</v>
@@ -39337,15 +39289,9 @@
       </c>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
-      <c r="G36" s="3">
-        <v>43.01</v>
-      </c>
-      <c r="H36" s="3">
-        <v>41.09</v>
-      </c>
-      <c r="I36" s="3">
-        <v>10</v>
-      </c>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
       <c r="J36" s="3">
         <v>43.21</v>
       </c>
@@ -40711,15 +40657,9 @@
       <c r="F55" s="3">
         <v>1.31</v>
       </c>
-      <c r="G55" s="3">
-        <v>41.32</v>
-      </c>
-      <c r="H55" s="3">
-        <v>29.88</v>
-      </c>
-      <c r="I55" s="3">
-        <v>5.39</v>
-      </c>
+      <c r="G55" s="3"/>
+      <c r="H55" s="3"/>
+      <c r="I55" s="3"/>
       <c r="J55" s="3">
         <v>0.01</v>
       </c>
@@ -41681,15 +41621,9 @@
       <c r="F68" s="3">
         <v>1.71</v>
       </c>
-      <c r="G68" s="3">
-        <v>31.26</v>
-      </c>
-      <c r="H68" s="3">
-        <v>20.43</v>
-      </c>
-      <c r="I68" s="3">
-        <v>6.14</v>
-      </c>
+      <c r="G68" s="3"/>
+      <c r="H68" s="3"/>
+      <c r="I68" s="3"/>
       <c r="J68" s="3">
         <v>0</v>
       </c>
@@ -42575,15 +42509,9 @@
       <c r="F80" s="3">
         <v>1.83</v>
       </c>
-      <c r="G80" s="3">
-        <v>6.76</v>
-      </c>
-      <c r="H80" s="3">
-        <v>4.6100000000000003</v>
-      </c>
-      <c r="I80" s="3">
-        <v>0</v>
-      </c>
+      <c r="G80" s="3"/>
+      <c r="H80" s="3"/>
+      <c r="I80" s="3"/>
       <c r="J80" s="3">
         <v>0.02</v>
       </c>
@@ -45047,7 +44975,7 @@
         <v>1050.7</v>
       </c>
       <c r="F5" s="5">
-        <v>17.899999999999999</v>
+        <v>34.8</v>
       </c>
       <c r="G5" s="5"/>
       <c r="H5" s="5">
@@ -46210,9 +46138,7 @@
       <c r="E12" s="5">
         <v>998.8</v>
       </c>
-      <c r="F12" s="5">
-        <v>28.96</v>
-      </c>
+      <c r="F12" s="5"/>
       <c r="G12" s="5"/>
       <c r="H12" s="5">
         <v>0.46</v>
@@ -46278,12 +46204,8 @@
       </c>
       <c r="AL12" s="3"/>
       <c r="AM12" s="3"/>
-      <c r="AN12" s="3">
-        <v>31.26</v>
-      </c>
-      <c r="AO12" s="3">
-        <v>5.65</v>
-      </c>
+      <c r="AN12" s="3"/>
+      <c r="AO12" s="3"/>
       <c r="AP12" s="3">
         <v>6.65</v>
       </c>
@@ -47751,7 +47673,7 @@
         <v>1050.3</v>
       </c>
       <c r="F5" s="5">
-        <v>31.72</v>
+        <v>51.92</v>
       </c>
       <c r="G5" s="5"/>
       <c r="H5" s="5">
@@ -48914,9 +48836,7 @@
       <c r="E12" s="5">
         <v>999.5</v>
       </c>
-      <c r="F12" s="5">
-        <v>35.33</v>
-      </c>
+      <c r="F12" s="5"/>
       <c r="G12" s="5"/>
       <c r="H12" s="5">
         <v>0.67</v>
@@ -48982,12 +48902,8 @@
       </c>
       <c r="AL12" s="3"/>
       <c r="AM12" s="3"/>
-      <c r="AN12" s="3">
-        <v>36.409999999999997</v>
-      </c>
-      <c r="AO12" s="3">
-        <v>8.23</v>
-      </c>
+      <c r="AN12" s="3"/>
+      <c r="AO12" s="3"/>
       <c r="AP12" s="3">
         <v>8.1999999999999993</v>
       </c>
@@ -50456,7 +50372,7 @@
         <v>1058.3</v>
       </c>
       <c r="F5" s="5">
-        <v>14.9</v>
+        <v>30.65</v>
       </c>
       <c r="G5" s="5"/>
       <c r="H5" s="5">
@@ -50524,10 +50440,10 @@
       <c r="AL5" s="3"/>
       <c r="AM5" s="3"/>
       <c r="AN5" s="3">
-        <v>32.869999999999997</v>
+        <v>36.56</v>
       </c>
       <c r="AO5" s="3">
-        <v>22.66</v>
+        <v>23.53</v>
       </c>
       <c r="AP5" s="3">
         <v>129.96</v>
@@ -51424,9 +51340,7 @@
       <c r="E11" s="5">
         <v>1016.1</v>
       </c>
-      <c r="F11" s="5">
-        <v>41.09</v>
-      </c>
+      <c r="F11" s="5"/>
       <c r="G11" s="5">
         <v>8.8000000000000078E-2</v>
       </c>
@@ -51496,12 +51410,8 @@
       </c>
       <c r="AL11" s="3"/>
       <c r="AM11" s="3"/>
-      <c r="AN11" s="3">
-        <v>43.01</v>
-      </c>
-      <c r="AO11" s="3">
-        <v>10</v>
-      </c>
+      <c r="AN11" s="3"/>
+      <c r="AO11" s="3"/>
       <c r="AP11" s="3">
         <v>43.21</v>
       </c>
@@ -54865,9 +54775,7 @@
       <c r="E15" s="5">
         <v>995.6</v>
       </c>
-      <c r="F15" s="5">
-        <v>29.88</v>
-      </c>
+      <c r="F15" s="5"/>
       <c r="G15" s="5">
         <v>9.220000000000006E-2</v>
       </c>
@@ -54939,12 +54847,8 @@
         <v>2.88</v>
       </c>
       <c r="AM15" s="3"/>
-      <c r="AN15" s="3">
-        <v>41.32</v>
-      </c>
-      <c r="AO15" s="3">
-        <v>5.39</v>
-      </c>
+      <c r="AN15" s="3"/>
+      <c r="AO15" s="3"/>
       <c r="AP15" s="3">
         <v>0.01</v>
       </c>
@@ -57212,9 +57116,7 @@
       <c r="E15" s="5">
         <v>994.5</v>
       </c>
-      <c r="F15" s="5">
-        <v>20.43</v>
-      </c>
+      <c r="F15" s="5"/>
       <c r="G15" s="5">
         <v>0.10299999999999976</v>
       </c>
@@ -57286,12 +57188,8 @@
         <v>2.88</v>
       </c>
       <c r="AM15" s="3"/>
-      <c r="AN15" s="3">
-        <v>31.26</v>
-      </c>
-      <c r="AO15" s="3">
-        <v>6.14</v>
-      </c>
+      <c r="AN15" s="3"/>
+      <c r="AO15" s="3"/>
       <c r="AP15" s="3">
         <v>0</v>
       </c>
@@ -59414,9 +59312,7 @@
       <c r="E14" s="5">
         <v>995.8</v>
       </c>
-      <c r="F14" s="5">
-        <v>4.6100000000000003</v>
-      </c>
+      <c r="F14" s="5"/>
       <c r="G14" s="5">
         <v>0.10789999999999988</v>
       </c>
@@ -59488,12 +59384,8 @@
         <v>2.86</v>
       </c>
       <c r="AM14" s="3"/>
-      <c r="AN14" s="3">
-        <v>6.76</v>
-      </c>
-      <c r="AO14" s="3">
-        <v>0</v>
-      </c>
+      <c r="AN14" s="3"/>
+      <c r="AO14" s="3"/>
       <c r="AP14" s="3">
         <v>0.02</v>
       </c>

</xml_diff>